<commit_message>
Updated to use event data
</commit_message>
<xml_diff>
--- a/DERT_Scouting_REBUILTTestData.xlsx
+++ b/DERT_Scouting_REBUILTTestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\JD Projects\DERT\QRCodeTest\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5D9F2A8-38FD-4A65-89DF-1A392BA644AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8546893D-DEF4-415B-8FAA-F4B41C4F2580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{5FC3C70B-391C-4AC5-A616-59B512FEB93E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{9C79E333-D847-466C-9963-53AC55AE0474}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -3773,49 +3773,49 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6B2E1984-65B5-40CE-AE0A-6A5E1B600691}" name="Scans" displayName="Scans" ref="A1:AN373" totalsRowShown="0" headerRowDxfId="7">
-  <autoFilter ref="A1:AN373" xr:uid="{6B2E1984-65B5-40CE-AE0A-6A5E1B600691}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0D8C34EF-4A3D-4EE6-84EC-0A9B0BF7A55D}" name="Scans" displayName="Scans" ref="A1:AN373" totalsRowShown="0" headerRowDxfId="7">
+  <autoFilter ref="A1:AN373" xr:uid="{0D8C34EF-4A3D-4EE6-84EC-0A9B0BF7A55D}"/>
   <tableColumns count="40">
-    <tableColumn id="1" xr3:uid="{165ADCF1-FACF-4E1F-96D9-EF1667ABBBB8}" name="Schema"/>
-    <tableColumn id="2" xr3:uid="{FB9DDC52-F98A-4FA0-8DFC-512D39BBB8BA}" name="Match type"/>
-    <tableColumn id="3" xr3:uid="{472C699B-360F-4CBA-B089-9E27B0FF921F}" name="Match #"/>
-    <tableColumn id="4" xr3:uid="{420026D5-104F-4CF3-B622-445C7AAD8C62}" name="Team #"/>
-    <tableColumn id="5" xr3:uid="{9EA3707D-FD29-4686-A872-35A4C5114768}" name="Alliance"/>
-    <tableColumn id="6" xr3:uid="{49CF85C7-7D2C-47AC-B936-913972EA7C40}" name="Station"/>
-    <tableColumn id="7" xr3:uid="{B36E3272-5A08-4F1D-9AB8-D3D44A4DB48A}" name="Scout name"/>
-    <tableColumn id="8" xr3:uid="{4E97710B-84AA-46E5-8DC8-779D06190057}" name="Robot on field?"/>
-    <tableColumn id="9" xr3:uid="{FEA54E7C-96B5-4244-9321-F329E81CAE85}" name="Starting position"/>
-    <tableColumn id="10" xr3:uid="{3236F85C-405E-4BCB-A1CE-7334BAB429BE}" name="Fuel preloaded"/>
-    <tableColumn id="11" xr3:uid="{129637A7-591B-4762-A8BC-51DF9C727F34}" name="Auto fuel scored"/>
-    <tableColumn id="12" xr3:uid="{E6C4F477-00E2-48C0-9F05-58CFC3AB2D8A}" name="Auto fuel missed"/>
-    <tableColumn id="13" xr3:uid="{1F07899D-71AC-4D63-96E8-8E0765826C9F}" name="Auto path"/>
-    <tableColumn id="14" xr3:uid="{156259D0-8F52-40BA-9BA4-B4CE69114ED1}" name="Picked up fuel from"/>
-    <tableColumn id="15" xr3:uid="{C0B31E2E-4D67-4013-AC42-03ACF8290734}" name="Tower climb in auto"/>
-    <tableColumn id="16" xr3:uid="{526644A6-7201-407F-B3AB-2DEEECCF7689}" name="Teleop fuel scored"/>
-    <tableColumn id="17" xr3:uid="{126B619B-8025-48D8-BD26-CDD6036A224A}" name="Teleop fuel missed"/>
-    <tableColumn id="18" xr3:uid="{F097CA7D-A20E-4E61-B268-63D50B8CF8E1}" name="Intake from"/>
-    <tableColumn id="19" xr3:uid="{8CC92FF3-FF62-4C0F-97A0-324BB8762E5B}" name="Shoots from"/>
-    <tableColumn id="20" xr3:uid="{4BB7E3E6-6538-446E-AED2-5DBD1C7178C4}" name="Drives over / through"/>
-    <tableColumn id="21" xr3:uid="{F721EDE3-8387-42DE-98B5-6547FE73A5BE}" name="Inactive Hub behavior"/>
-    <tableColumn id="22" xr3:uid="{0B1CEDCD-7CA2-4B68-B2D3-F3EB28DB7E6E}" name="Fuel it can carry"/>
-    <tableColumn id="23" xr3:uid="{BD028730-6360-4EFF-A255-E7D1ED341732}" name="Played defense"/>
-    <tableColumn id="24" xr3:uid="{1829728B-FB25-4646-81B0-A6B9B99D47A3}" name="Was defended"/>
-    <tableColumn id="25" xr3:uid="{6E70FAE5-C564-4FFF-B060-760B45008ED4}" name="Tower climb"/>
-    <tableColumn id="26" xr3:uid="{56C78450-EAAB-4F4B-ACFE-339DF5296136}" name="Climb time"/>
-    <tableColumn id="27" xr3:uid="{3ACE48A1-802E-4CBC-B577-0C5B2A11F673}" name="Driver skill"/>
-    <tableColumn id="28" xr3:uid="{40F17BDC-5B05-4477-A062-2069ABC2259D}" name="Robot speed"/>
-    <tableColumn id="29" xr3:uid="{A0A34485-5517-45EC-92C3-C04E664AC62D}" name="Shooting accuracy"/>
-    <tableColumn id="30" xr3:uid="{128E2542-C424-4191-8873-4CBF7901D2A4}" name="Problems"/>
-    <tableColumn id="31" xr3:uid="{18C1FD10-6E9A-4CC7-A815-C7CD0D389D8D}" name="Minor fouls"/>
-    <tableColumn id="32" xr3:uid="{B5099AD8-8636-471A-B77D-E554E185EAE3}" name="Major fouls"/>
-    <tableColumn id="33" xr3:uid="{766C191F-A961-4CC1-874F-2570804426C1}" name="Card"/>
-    <tableColumn id="34" xr3:uid="{5DBADD42-CE17-475A-A96D-0DEFB96AA5EF}" name="Pick?"/>
-    <tableColumn id="35" xr3:uid="{AE1725AE-DD47-4BD9-BE87-943004C17D38}" name="Observations"/>
-    <tableColumn id="36" xr3:uid="{1958EE53-ECE4-44C1-84E4-A503C531C816}" name="Auto pts" dataDxfId="6"/>
-    <tableColumn id="37" xr3:uid="{214616B7-32AF-4DA7-9F21-79603082F721}" name="Teleop fuel pts" dataDxfId="5"/>
-    <tableColumn id="38" xr3:uid="{1B431953-A2D9-49FB-9A36-7E281DE201BC}" name="Climb pts" dataDxfId="4"/>
-    <tableColumn id="39" xr3:uid="{78CFCB0D-9D96-4EF6-9D32-207784BAA452}" name="Total pts" dataDxfId="3"/>
-    <tableColumn id="40" xr3:uid="{FFD9632E-7763-4184-B822-2856735452C1}" name="Submitted"/>
+    <tableColumn id="1" xr3:uid="{9FD3F422-3B72-41AB-BE3F-C9213416EC50}" name="Schema"/>
+    <tableColumn id="2" xr3:uid="{14C9E7ED-6635-4FA2-94DD-F0184A4497B1}" name="Match type"/>
+    <tableColumn id="3" xr3:uid="{0004BB5C-7F98-4FD5-87C2-1DCB30F0742A}" name="Match #"/>
+    <tableColumn id="4" xr3:uid="{1D2338C8-AF45-4C0C-9D25-BC23FFE46B0C}" name="Team #"/>
+    <tableColumn id="5" xr3:uid="{9720B775-ACC3-4FD3-842D-56E60DF8CA3F}" name="Alliance"/>
+    <tableColumn id="6" xr3:uid="{0B646EC8-208C-42D1-A49E-23D26798283B}" name="Station"/>
+    <tableColumn id="7" xr3:uid="{5FA49D8F-1100-44F2-A1E4-CF4A6D815AAA}" name="Scout name"/>
+    <tableColumn id="8" xr3:uid="{7FDD5858-F1D3-432E-B75B-F8710F545AF0}" name="Robot on field?"/>
+    <tableColumn id="9" xr3:uid="{231F0FCD-FD19-491E-B12F-168717EC9943}" name="Starting position"/>
+    <tableColumn id="10" xr3:uid="{25DF6EDA-1D7D-4DBB-BD08-9BC5259626BB}" name="Fuel preloaded"/>
+    <tableColumn id="11" xr3:uid="{4BD818AD-AECA-4CE5-A591-B4EFDAC0DD98}" name="Auto fuel scored"/>
+    <tableColumn id="12" xr3:uid="{3440292F-45C9-4C08-B343-4A27C9CDD58B}" name="Auto fuel missed"/>
+    <tableColumn id="13" xr3:uid="{92235D31-8610-48E3-9143-2171F2BA56A6}" name="Auto path"/>
+    <tableColumn id="14" xr3:uid="{04B56BF7-BF3C-459B-BA9F-9AB5F5F13443}" name="Picked up fuel from"/>
+    <tableColumn id="15" xr3:uid="{C1CC9C2C-A7DB-4CC5-87DE-6903712568D5}" name="Tower climb in auto"/>
+    <tableColumn id="16" xr3:uid="{1670C1C1-32E2-4D9F-A372-C30CB056A369}" name="Teleop fuel scored"/>
+    <tableColumn id="17" xr3:uid="{50FD596B-2541-446C-B763-852B5A936194}" name="Teleop fuel missed"/>
+    <tableColumn id="18" xr3:uid="{CC731CD5-7BE7-4244-8B9D-EED15758DA46}" name="Intake from"/>
+    <tableColumn id="19" xr3:uid="{EBA68361-BD2D-4ED0-8EC8-0DD4EA8E5C10}" name="Shoots from"/>
+    <tableColumn id="20" xr3:uid="{A24C8CBC-CEBB-4BD4-B600-CBBDAF036849}" name="Drives over / through"/>
+    <tableColumn id="21" xr3:uid="{36F5B4F7-C988-4659-8262-AB2CAFB74DA7}" name="Inactive Hub behavior"/>
+    <tableColumn id="22" xr3:uid="{8A5BA21C-3DE5-4054-BB72-F0B21BFF376B}" name="Fuel it can carry"/>
+    <tableColumn id="23" xr3:uid="{38ECAD4A-D25D-43E3-831D-47B9AA56EE68}" name="Played defense"/>
+    <tableColumn id="24" xr3:uid="{D55507DA-A3AC-4567-88D6-4E805C0444F1}" name="Was defended"/>
+    <tableColumn id="25" xr3:uid="{532D9111-B321-4D9D-9AF8-805E5F6FFD72}" name="Tower climb"/>
+    <tableColumn id="26" xr3:uid="{E90DE189-222F-4F66-9503-E04D6059E109}" name="Climb time"/>
+    <tableColumn id="27" xr3:uid="{48E4655B-E882-4986-BC08-55ECF322006A}" name="Driver skill"/>
+    <tableColumn id="28" xr3:uid="{5AC21FF9-BB70-4E24-B990-00D89A4E2C23}" name="Robot speed"/>
+    <tableColumn id="29" xr3:uid="{02C81584-1F66-4225-A8BD-BB0765F5EE73}" name="Shooting accuracy"/>
+    <tableColumn id="30" xr3:uid="{570DA32F-A386-4312-B413-2F55DB0564CA}" name="Problems"/>
+    <tableColumn id="31" xr3:uid="{F61D8F99-C4FE-4ED8-BBE0-CAB5AB531F96}" name="Minor fouls"/>
+    <tableColumn id="32" xr3:uid="{45ED257A-2E8F-4998-B7B4-A6A77CC5972B}" name="Major fouls"/>
+    <tableColumn id="33" xr3:uid="{8B101E37-BC0C-4A95-A009-67528AC3A895}" name="Card"/>
+    <tableColumn id="34" xr3:uid="{27A923BA-908D-4FFF-9E1E-4386D8E20B34}" name="Pick?"/>
+    <tableColumn id="35" xr3:uid="{BCAD94F2-A580-4C88-9B62-9024F6F14FDE}" name="Observations"/>
+    <tableColumn id="36" xr3:uid="{0A42537D-0E3A-4C7E-B314-E4C5DDDDB080}" name="Auto pts" dataDxfId="6"/>
+    <tableColumn id="37" xr3:uid="{0A026D85-5C26-4FE4-9A93-1EFEAF0A6B45}" name="Teleop fuel pts" dataDxfId="5"/>
+    <tableColumn id="38" xr3:uid="{0198F8C5-A982-44E8-89D2-E567E3FE50F1}" name="Climb pts" dataDxfId="4"/>
+    <tableColumn id="39" xr3:uid="{9BA3FC45-30EF-4F43-A548-0CD30EFA3C08}" name="Total pts" dataDxfId="3"/>
+    <tableColumn id="40" xr3:uid="{37813D61-A455-41B9-AE13-7E089FC29B12}" name="Submitted"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4137,7 +4137,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1070122C-F992-4DD7-997E-6DE3E0076B37}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DB0A9BD-D696-40F8-87B5-83D79FB5A553}">
   <dimension ref="A1:J89"/>
   <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4645,7 +4645,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75B10AE2-B3EF-43C4-8B88-2CBC5E6550F0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E829ADA5-22E5-4A13-A739-C8A0C23742A5}">
   <dimension ref="A1:AN373"/>
   <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
@@ -46779,7 +46779,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3F53B4E-5463-4B3B-BD99-979AF0DB8078}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CAA8B9B-35FE-4FD5-AE48-8038D241A052}">
   <dimension ref="A1:AC304"/>
   <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
@@ -57757,7 +57757,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2463A32-11E1-43DB-AA24-6AE44966559D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E0B4CE6-F39C-442F-85B2-D77C7653AA6D}">
   <dimension ref="A1:AN17"/>
   <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
@@ -59421,7 +59421,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{106A1ACA-B1D7-4789-BC81-624AEBFBA0CD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03920870-E7B9-4885-A83D-80006FFD5B2E}">
   <dimension ref="A1:G3000"/>
   <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
@@ -77525,7 +77525,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18C0EF48-655C-422C-ADB4-F7A56922F04D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48C94EC1-2037-4C39-8ED3-75A96A679356}">
   <dimension ref="A1:T473"/>
   <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
@@ -77612,7 +77612,7 @@
         <v>4</v>
       </c>
       <c r="R5" cm="1">
-        <f t="array" ref="R5:T376">_xlfn.LET(_xlpm.src,A1:H2000,_xlpm.a,INDEX(_xlpm.src,,1),_xlpm.line,IF(INDEX(_xlpm.src,,2)="",_xlpm.a,_xlpm.a&amp;","&amp;INDEX(_xlpm.src,,2)&amp;","&amp;INDEX(_xlpm.src,,3)&amp;","&amp;INDEX(_xlpm.src,,4)&amp;","&amp;INDEX(_xlpm.src,,5)&amp;","&amp;INDEX(_xlpm.src,,6)&amp;","&amp;INDEX(_xlpm.src,,7)&amp;","&amp;INDEX(_xlpm.src,,8)),_xlpm.t,","&amp;_xlpm.line&amp;",",_xlpm.lvl,IFERROR(_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(_xlpm.t,",",4),","),""),_xlpm.num,IFERROR(--_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(_xlpm.t,",",5),","),""),_xlpm.side,LOWER(IFERROR(_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(_xlpm.t,",",7),","),"")),_xlpm.tm,IFERROR(--_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(_xlpm.t,",",8),","),""),_xlpm.keep,ISNUMBER(_xlpm.num)*ISNUMBER(_xlpm.tm)*(_xlpm.lvl="qm")*((_xlpm.side="red")+(_xlpm.side="blue")),IFERROR(_xlfn._xlws.FILTER(_xlfn.HSTACK(_xlpm.num,PROPER(_xlpm.side),_xlpm.tm),_xlpm.keep),_xlfn.HSTACK("","","")))</f>
+        <f t="array" ref="R5:T376">_xlfn.LET(_xlpm.src,A1:H2000,_xlpm.a,INDEX(_xlpm.src,,1),_xlpm.line,IF(INDEX(_xlpm.src,,2)="",_xlpm.a,_xlpm.a&amp;","&amp;INDEX(_xlpm.src,,2)&amp;","&amp;INDEX(_xlpm.src,,3)&amp;","&amp;INDEX(_xlpm.src,,4)&amp;","&amp;INDEX(_xlpm.src,,5)&amp;","&amp;INDEX(_xlpm.src,,6)&amp;","&amp;INDEX(_xlpm.src,,7)&amp;","&amp;INDEX(_xlpm.src,,8)),_xlpm.t,","&amp;_xlpm.line&amp;",",_xlpm.lvl,IFERROR(_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(_xlpm.t,",",4),","),""),_xlpm.num,IFERROR(--_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(_xlpm.t,",",5),","),""),_xlpm.side,LOWER(IFERROR(_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(_xlpm.t,",",7),","),"")),_xlpm.tr,IFERROR(_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(_xlpm.t,",",8),","),""),_xlpm.tm,IFERROR(--_xlpm.tr,UPPER(_xlpm.tr)),_xlpm.keep,ISNUMBER(_xlpm.num)*(_xlpm.tr&lt;&gt;"")*(_xlpm.lvl="qm")*((_xlpm.side="red")+(_xlpm.side="blue")),IFERROR(_xlfn._xlws.FILTER(_xlfn.HSTACK(_xlpm.num,PROPER(_xlpm.side),_xlpm.tm),_xlpm.keep),_xlfn.HSTACK("","","")))</f>
         <v>1</v>
       </c>
       <c r="S5" t="str">
@@ -83322,7 +83322,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70F71AB1-44CC-4141-99A1-590F34F3C90D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CC9BBF3-EF22-40C3-B17D-EB6E430B815A}">
   <dimension ref="A1:S36"/>
   <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>